<commit_message>
Improve Master patrol config
</commit_message>
<xml_diff>
--- a/storage/template/TEMPLATE-KONFIGURASI-PATROLI.xlsx
+++ b/storage/template/TEMPLATE-KONFIGURASI-PATROLI.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imamsyz/PhpstormProjects/digipatrol-v2/storage/template-doc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/imamsyz/PhpstormProjects/digipatrol.id/storage/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69BC220B-E450-964D-ABD7-0315AC4EAA8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DCBDAE-2C68-674A-ABC5-27EFBC9E7FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1820" yWindow="3540" windowWidth="29860" windowHeight="15420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1240" yWindow="-21600" windowWidth="38400" windowHeight="21600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE KATEGORI" sheetId="1" r:id="rId1"/>
     <sheet name="SAMPLE DATA" sheetId="2" r:id="rId2"/>
     <sheet name="KATEGORI" sheetId="3" r:id="rId3"/>
-    <sheet name="DATA" sheetId="4" r:id="rId4"/>
+    <sheet name="EVENT KATEGORI" sheetId="5" r:id="rId4"/>
+    <sheet name="DATA" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="102">
   <si>
     <t>NO</t>
   </si>
@@ -315,13 +316,40 @@
   </si>
   <si>
     <t>KODE_NFC</t>
+  </si>
+  <si>
+    <t>EVENT</t>
+  </si>
+  <si>
+    <t>MATI</t>
+  </si>
+  <si>
+    <t>KONSLET</t>
+  </si>
+  <si>
+    <t>PECAH</t>
+  </si>
+  <si>
+    <t>HILANG</t>
+  </si>
+  <si>
+    <t>KATEGORI</t>
+  </si>
+  <si>
+    <t>RUSAK</t>
+  </si>
+  <si>
+    <t>BOCOR</t>
+  </si>
+  <si>
+    <t>LAINNYA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -357,8 +385,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -401,6 +441,12 @@
         <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -414,7 +460,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -454,6 +500,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -543,11 +590,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table_2" displayName="Table_2" ref="A2:C6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table_2" displayName="Table_2" ref="A1:C5">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="NO"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="KODE KATEGORI"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="NAMA_KATEGORI"/>
+  </tableColumns>
+  <tableStyleInfo name="KATEGORI-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A003C2DA-ED3C-9341-9C66-A8D9D4C6C9F5}" name="Table_24" displayName="Table_24" ref="A1:C16">
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{55FD2C56-79BE-0B48-8A22-A1E9A6FABFEB}" name="KODE"/>
+    <tableColumn id="3" xr3:uid="{CD1A318F-88C9-0347-B0CC-CF3E6ED68886}" name="KATEGORI"/>
+    <tableColumn id="2" xr3:uid="{20A0AE87-9DB2-9243-9435-90BC5C1825A5}" name="EVENT"/>
   </tableColumns>
   <tableStyleInfo name="KATEGORI-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -942,7 +1000,7 @@
       </c>
       <c r="E9" s="14">
         <f ca="1">RANDBETWEEN(1000000,99999999)</f>
-        <v>42404233</v>
+        <v>70113115</v>
       </c>
       <c r="F9" s="13"/>
     </row>
@@ -1139,7 +1197,7 @@
       <c r="D20" s="13"/>
       <c r="E20" s="14">
         <f ca="1">RANDBETWEEN(1000000,99999999)</f>
-        <v>99880815</v>
+        <v>48086528</v>
       </c>
       <c r="F20" s="13"/>
     </row>
@@ -1350,7 +1408,7 @@
       <c r="D32" s="13"/>
       <c r="E32" s="17">
         <f ca="1">RANDBETWEEN(1000000,99999999)</f>
-        <v>15340927</v>
+        <v>99685455</v>
       </c>
       <c r="F32" s="13"/>
     </row>
@@ -4322,7 +4380,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A2:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5.33203125" customWidth="1"/>
@@ -4330,58 +4388,58 @@
     <col min="3" max="3" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="2">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -4394,11 +4452,150 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE72A205-E79F-F54F-80FD-654B06AC6B60}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A2" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A3" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A4" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A5" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A6" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A5:G5"/>
+  <dimension ref="A3:G39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -4408,6 +4605,14 @@
     <col min="9" max="9" width="25.1640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
     <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="5" t="s">
         <v>13</v>
@@ -4429,7 +4634,620 @@
       </c>
       <c r="G5" s="3"/>
     </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="7">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="8"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="9">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="11">
+        <v>3</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="11"/>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="13">
+        <v>4</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="14">
+        <f ca="1">RANDBETWEEN(1000000,99999999)</f>
+        <v>62199219</v>
+      </c>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="15">
+        <v>5</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="F10" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="15">
+        <v>5</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="15">
+        <v>5</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="16"/>
+      <c r="F12" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="15">
+        <v>5</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="15">
+        <v>5</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="15">
+        <v>5</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="F15" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="15">
+        <v>5</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="16"/>
+      <c r="F16" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="15">
+        <v>5</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="16"/>
+      <c r="F17" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="15">
+        <v>5</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="16"/>
+      <c r="F18" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="15">
+        <v>5</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="16"/>
+      <c r="F19" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="13">
+        <v>4</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="14">
+        <f ca="1">RANDBETWEEN(1000000,99999999)</f>
+        <v>22729443</v>
+      </c>
+      <c r="F20" s="13"/>
+    </row>
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="15">
+        <v>5</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="15">
+        <v>5</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E22" s="16"/>
+      <c r="F22" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="15">
+        <v>5</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="16"/>
+      <c r="F23" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="15">
+        <v>5</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="16"/>
+      <c r="F24" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="15">
+        <v>5</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" s="16"/>
+      <c r="F25" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="15">
+        <v>5</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="16"/>
+      <c r="F26" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="15">
+        <v>5</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" s="16"/>
+      <c r="F27" s="15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="15">
+        <v>5</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="15">
+        <v>5</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" s="16"/>
+      <c r="F29" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="15">
+        <v>5</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" s="16"/>
+      <c r="F30" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="11">
+        <v>3</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="11"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="11"/>
+    </row>
+    <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="13">
+        <v>4</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D32" s="13"/>
+      <c r="E32" s="17">
+        <f ca="1">RANDBETWEEN(1000000,99999999)</f>
+        <v>5897578</v>
+      </c>
+      <c r="F32" s="13"/>
+    </row>
+    <row r="33" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="15">
+        <v>5</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33" s="18"/>
+      <c r="F33" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A34" s="15">
+        <v>5</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="18"/>
+      <c r="F34" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="15">
+        <v>5</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E35" s="18"/>
+      <c r="F35" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A36" s="15">
+        <v>5</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36" s="18"/>
+      <c r="F36" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="15">
+        <v>5</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E37" s="18"/>
+      <c r="F37" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="15">
+        <v>5</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E38" s="18"/>
+      <c r="F38" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A39" s="15">
+        <v>5</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E39" s="18"/>
+      <c r="F39" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{FE1F03AF-9475-4141-B32C-8E33D2577437}">
+          <x14:formula1>
+            <xm:f>'SAMPLE KATEGORI'!$C$3:$C$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>F10:F19 F21:F30 F33:F39</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>